<commit_message>
Repeater prototype wiring diagram (PCB v4.0 harness) + shopping list extras
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PGMYLJZdJJDWKnHJD8ynzD
</commit_message>
<xml_diff>
--- a/hardware/repeater_x2_shopping_list.xlsx
+++ b/hardware/repeater_x2_shopping_list.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="79">
   <si>
     <t xml:space="preserve">MineSafe — components for 2 repeaters (PCB v4.0 + case)</t>
   </si>
@@ -175,7 +175,28 @@
     <t xml:space="preserve">Optional for demo</t>
   </si>
   <si>
-    <t xml:space="preserve">12 V 2 A adapter (mine-supply stand-in)</t>
+    <t xml:space="preserve">DC adapter 15–24 V, 2 A (mine-supply stand-in)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 V ideal: supply then wins over the battery (see wiring diagram)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wago 221-413 lever splitter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 per box: splits supply to J1 + charge module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inline 3 A blade fuse holder + fuse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In battery P+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wire: 0.75 mm² red/black 2 m, 26 AWG 6 colours, Dupont housings, heat-shrink</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lot for both boxes</t>
   </si>
   <si>
     <t xml:space="preserve">22 mm IP67 red mushroom button (SOS)</t>
@@ -238,7 +259,7 @@
     <t xml:space="preserve">• For the demo you can skip the battery packs and run off the 12 V adapters.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Full details: hardware/README.md and hardware/repeater_pcb/bom_pcb.csv in the MINESAFE repo.</t>
+    <t xml:space="preserve">• Wiring: docs/wiring/repeater_v4_wiring.png. Full details: hardware/README.md and hardware/repeater_pcb/bom_pcb.csv in the MINESAFE repo.</t>
   </si>
 </sst>
 </file>
@@ -801,7 +822,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -1623,120 +1644,126 @@
         <v>2</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="D38" s="11" t="n">
         <f aca="false">B38*C38</f>
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="E38" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F38" s="11" t="n">
         <f aca="false">IF(UPPER(E38)="Y",0,D38)</f>
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="G38" s="12"/>
       <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
+      <c r="I38" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B39" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C39" s="10" t="n">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="D39" s="11" t="n">
         <f aca="false">B39*C39</f>
-        <v>300</v>
+        <v>160</v>
       </c>
       <c r="E39" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F39" s="11" t="n">
         <f aca="false">IF(UPPER(E39)="Y",0,D39)</f>
-        <v>300</v>
+        <v>160</v>
       </c>
       <c r="G39" s="12"/>
       <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
+      <c r="I39" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B40" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C40" s="10" t="n">
-        <v>250</v>
+        <v>40</v>
       </c>
       <c r="D40" s="11" t="n">
         <f aca="false">B40*C40</f>
-        <v>500</v>
+        <v>80</v>
       </c>
       <c r="E40" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F40" s="11" t="n">
         <f aca="false">IF(UPPER(E40)="Y",0,D40)</f>
-        <v>500</v>
+        <v>80</v>
       </c>
       <c r="G40" s="12"/>
       <c r="H40" s="8"/>
-      <c r="I40" s="8"/>
+      <c r="I40" s="8" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="8" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B41" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C41" s="10" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D41" s="11" t="n">
         <f aca="false">B41*C41</f>
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E41" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F41" s="11" t="n">
         <f aca="false">IF(UPPER(E41)="Y",0,D41)</f>
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G41" s="12"/>
       <c r="H41" s="8"/>
       <c r="I41" s="8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B42" s="9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="D42" s="11" t="n">
         <f aca="false">B42*C42</f>
-        <v>360</v>
+        <v>300</v>
       </c>
       <c r="E42" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F42" s="11" t="n">
         <f aca="false">IF(UPPER(E42)="Y",0,D42)</f>
-        <v>360</v>
+        <v>300</v>
       </c>
       <c r="G42" s="12"/>
       <c r="H42" s="8"/>
@@ -1744,24 +1771,24 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B43" s="9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C43" s="10" t="n">
-        <v>30</v>
+        <v>250</v>
       </c>
       <c r="D43" s="11" t="n">
         <f aca="false">B43*C43</f>
-        <v>240</v>
+        <v>500</v>
       </c>
       <c r="E43" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F43" s="11" t="n">
         <f aca="false">IF(UPPER(E43)="Y",0,D43)</f>
-        <v>240</v>
+        <v>500</v>
       </c>
       <c r="G43" s="12"/>
       <c r="H43" s="8"/>
@@ -1769,49 +1796,51 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B44" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C44" s="10" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="D44" s="11" t="n">
         <f aca="false">B44*C44</f>
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="E44" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F44" s="11" t="n">
         <f aca="false">IF(UPPER(E44)="Y",0,D44)</f>
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="G44" s="12"/>
       <c r="H44" s="8"/>
-      <c r="I44" s="8"/>
+      <c r="I44" s="8" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B45" s="9" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C45" s="10" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="D45" s="11" t="n">
         <f aca="false">B45*C45</f>
-        <v>96</v>
+        <v>360</v>
       </c>
       <c r="E45" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F45" s="11" t="n">
         <f aca="false">IF(UPPER(E45)="Y",0,D45)</f>
-        <v>96</v>
+        <v>360</v>
       </c>
       <c r="G45" s="12"/>
       <c r="H45" s="8"/>
@@ -1819,24 +1848,24 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B46" s="9" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C46" s="10" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="D46" s="11" t="n">
         <f aca="false">B46*C46</f>
-        <v>84</v>
+        <v>240</v>
       </c>
       <c r="E46" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F46" s="11" t="n">
         <f aca="false">IF(UPPER(E46)="Y",0,D46)</f>
-        <v>84</v>
+        <v>240</v>
       </c>
       <c r="G46" s="12"/>
       <c r="H46" s="8"/>
@@ -1844,51 +1873,49 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B47" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C47" s="10" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="D47" s="11" t="n">
         <f aca="false">B47*C47</f>
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="E47" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F47" s="11" t="n">
         <f aca="false">IF(UPPER(E47)="Y",0,D47)</f>
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="G47" s="12"/>
       <c r="H47" s="8"/>
-      <c r="I47" s="8" t="s">
-        <v>61</v>
-      </c>
+      <c r="I47" s="8"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B48" s="9" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C48" s="10" t="n">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="D48" s="11" t="n">
         <f aca="false">B48*C48</f>
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E48" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F48" s="11" t="n">
         <f aca="false">IF(UPPER(E48)="Y",0,D48)</f>
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="G48" s="12"/>
       <c r="H48" s="8"/>
@@ -1896,136 +1923,213 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B49" s="9" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C49" s="10" t="n">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="D49" s="11" t="n">
         <f aca="false">B49*C49</f>
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E49" s="12" t="s">
         <v>13</v>
       </c>
       <c r="F49" s="11" t="n">
         <f aca="false">IF(UPPER(E49)="Y",0,D49)</f>
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="G49" s="12"/>
       <c r="H49" s="8"/>
-      <c r="I49" s="8" t="s">
-        <v>64</v>
-      </c>
+      <c r="I49" s="8"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="B50" s="14"/>
-      <c r="C50" s="15"/>
-      <c r="D50" s="15" t="n">
-        <f aca="false">SUM(D36:D49)</f>
-        <v>6700</v>
-      </c>
-      <c r="E50" s="14"/>
-      <c r="F50" s="15" t="n">
-        <f aca="false">SUM(F36:F49)</f>
-        <v>6700</v>
-      </c>
-      <c r="G50" s="14"/>
-      <c r="H50" s="13"/>
-      <c r="I50" s="13"/>
+      <c r="A50" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B50" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="D50" s="11" t="n">
+        <f aca="false">B50*C50</f>
+        <v>120</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" s="11" t="n">
+        <f aca="false">IF(UPPER(E50)="Y",0,D50)</f>
+        <v>120</v>
+      </c>
+      <c r="G50" s="12"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="8" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="16"/>
-      <c r="B51" s="17"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="17"/>
-      <c r="F51" s="18"/>
-      <c r="G51" s="17"/>
-      <c r="H51" s="16"/>
-      <c r="I51" s="16"/>
+      <c r="A51" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B51" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="D51" s="11" t="n">
+        <f aca="false">B51*C51</f>
+        <v>120</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="11" t="n">
+        <f aca="false">IF(UPPER(E51)="Y",0,D51)</f>
+        <v>120</v>
+      </c>
+      <c r="G51" s="12"/>
+      <c r="H51" s="8"/>
+      <c r="I51" s="8"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="B52" s="20"/>
-      <c r="C52" s="21"/>
-      <c r="D52" s="21" t="n">
-        <f aca="false">D13+D33+D50</f>
-        <v>12984</v>
-      </c>
-      <c r="E52" s="20"/>
-      <c r="F52" s="21" t="n">
-        <f aca="false">F13+F33+F50</f>
-        <v>12984</v>
-      </c>
-      <c r="G52" s="20"/>
-      <c r="H52" s="19"/>
-      <c r="I52" s="19"/>
+      <c r="A52" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B52" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="D52" s="11" t="n">
+        <f aca="false">B52*C52</f>
+        <v>100</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" s="11" t="n">
+        <f aca="false">IF(UPPER(E52)="Y",0,D52)</f>
+        <v>100</v>
+      </c>
+      <c r="G52" s="12"/>
+      <c r="H52" s="8"/>
+      <c r="I52" s="8" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="22" t="s">
-        <v>67</v>
-      </c>
-      <c r="B53" s="23"/>
-      <c r="C53" s="24"/>
-      <c r="D53" s="24" t="n">
-        <f aca="false">D52/2</f>
-        <v>6492</v>
-      </c>
-      <c r="E53" s="23"/>
-      <c r="F53" s="24" t="n">
-        <f aca="false">F52/2</f>
-        <v>6492</v>
-      </c>
-      <c r="G53" s="23"/>
-      <c r="H53" s="22"/>
-      <c r="I53" s="22"/>
+      <c r="A53" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B53" s="14"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="15" t="n">
+        <f aca="false">SUM(D36:D52)</f>
+        <v>7440</v>
+      </c>
+      <c r="E53" s="14"/>
+      <c r="F53" s="15" t="n">
+        <f aca="false">SUM(F36:F52)</f>
+        <v>7440</v>
+      </c>
+      <c r="G53" s="14"/>
+      <c r="H53" s="13"/>
+      <c r="I53" s="13"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="16"/>
+      <c r="B54" s="17"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="17"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="17"/>
+      <c r="H54" s="16"/>
+      <c r="I54" s="16"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="25" t="s">
+      <c r="A55" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="B55" s="20"/>
+      <c r="C55" s="21"/>
+      <c r="D55" s="21" t="n">
+        <f aca="false">D13+D33+D53</f>
+        <v>13724</v>
+      </c>
+      <c r="E55" s="20"/>
+      <c r="F55" s="21" t="n">
+        <f aca="false">F13+F33+F53</f>
+        <v>13724</v>
+      </c>
+      <c r="G55" s="20"/>
+      <c r="H55" s="19"/>
+      <c r="I55" s="19"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B56" s="23"/>
+      <c r="C56" s="24"/>
+      <c r="D56" s="24" t="n">
+        <f aca="false">D55/2</f>
+        <v>6862</v>
+      </c>
+      <c r="E56" s="23"/>
+      <c r="F56" s="24" t="n">
+        <f aca="false">F55/2</f>
+        <v>6862</v>
+      </c>
+      <c r="G56" s="23"/>
+      <c r="H56" s="22"/>
+      <c r="I56" s="22"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="25" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="26" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="26" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="26" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="26" t="s">
-        <v>71</v>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="26" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="26" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="26" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A6:I50">
+  <conditionalFormatting sqref="A6:I53">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$G6="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E6:E12 E16:E32 E36:E49" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E6:E12 E16:E32 E36:E52" type="list">
       <formula1>"Y,N"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G6:G12 G16:G32 G36:G49" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G6:G12 G16:G32 G36:G52" type="list">
       <formula1>"✓"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>